<commit_message>
add 2023 NEI data and re-run all
</commit_message>
<xml_diff>
--- a/_transportation/data-raw/epa/epa_downloads.xlsx
+++ b/_transportation/data-raw/epa/epa_downloads.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rotenle/Documents/MetC_Locals/Interdivisional/ghg-cprg/_transportation/data-raw/epa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E53FCC88-E2B5-1645-9BA1-FC36B2D09720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8264196E-86BF-2F4B-A5E5-D354F50E818D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3840" yWindow="900" windowWidth="30720" windowHeight="17040" xr2:uid="{E3501ACA-8D46-AF4B-AC5D-95BB483C9130}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1264" uniqueCount="354">
   <si>
     <t>file_name</t>
   </si>
@@ -1028,6 +1028,81 @@
   </si>
   <si>
     <t>https://gaftp.epa.gov/Air/nei/2008/flat_files/2008NEIv3_POINT_20130206.zip</t>
+  </si>
+  <si>
+    <t>2023NEI</t>
+  </si>
+  <si>
+    <t>_transportation/data-raw/epa/nei/2023NEI</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/flat_files/SmokeFlatFile_ONROAD_20260420.zip</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/onroad/2023NEI_onroad_activity_final_20251010.zip</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/onroad/2023_Documentation_of_CDB_Input_Data_20251013.xlsx</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/onroad/2022-2023_StreetLight_Grouping_Decision_Charts.pdf</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/onroad/2023NEI_default_onroad_activity_approach.pdf</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/onroad/CDBs_for_all_counties/2023_CDBs_state55.zip</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/onroad/CDBs_for_all_counties/2023_CDBs_state27.zip</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/data_summaries/2023nei_nonroad_byregion.zip</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/data_summaries/2023nei_onroad_byregion.zip</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/nonroad/nonroad_equipment_emissions_comparison_2023NEI_draft_2022hd.xlsx</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/onroad/2023NEI_RepCounty_Temperatures.zip</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/onroad/2023_Representative_Counties_Analysis_20250530.xlsx</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/data_summaries/eis_report_37532_county_Sector_allpolls_19may26.zip</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/flat_files/SmokeFlatFile_POINT_20260515.zip</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/point/Airports/2023-NEI-Aviation-Documentation_Final.pdf</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/point/Airports/2023-lead-calculations-by-state-final.xlsx</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/point/Airports/2023-lead-calculations-by-state-final.pdf</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/nonroad/inputs/2023NonroadSCCaggregation.xlsx</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/nonroad/inputs/2023_NonroadCDBs.zip</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/point/tagged_SLTdata_2023NEI_19may2026.csv</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/Air/nei/2023/doc/supporting_data/point/2023_point_defaultMax_poll_thresholds_qa_01May2026.csv</t>
+  </si>
+  <si>
+    <t>https://gaftp.epa.gov/air/nei/2023/data_summaries/eis_report_37583_2023NEI_facility_summary.zip</t>
   </si>
 </sst>
 </file>
@@ -1618,7 +1693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB8EF959-18DF-BD43-B878-2D065289D72D}">
-  <dimension ref="A1:I193"/>
+  <dimension ref="A1:I215"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.6640625" customWidth="1"/>
@@ -6097,6 +6172,509 @@
       </c>
       <c r="I193" t="s">
         <v>328</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A194" t="s">
+        <v>72</v>
+      </c>
+      <c r="B194">
+        <v>2023</v>
+      </c>
+      <c r="C194" t="s">
+        <v>237</v>
+      </c>
+      <c r="D194" t="s">
+        <v>9</v>
+      </c>
+      <c r="F194" t="s">
+        <v>329</v>
+      </c>
+      <c r="H194" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I194" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A195" t="s">
+        <v>72</v>
+      </c>
+      <c r="B195">
+        <v>2023</v>
+      </c>
+      <c r="C195" t="s">
+        <v>49</v>
+      </c>
+      <c r="D195" t="s">
+        <v>9</v>
+      </c>
+      <c r="F195" t="s">
+        <v>329</v>
+      </c>
+      <c r="H195" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I195" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A196" t="s">
+        <v>72</v>
+      </c>
+      <c r="B196">
+        <v>2023</v>
+      </c>
+      <c r="C196" t="s">
+        <v>170</v>
+      </c>
+      <c r="D196" t="s">
+        <v>9</v>
+      </c>
+      <c r="F196" t="s">
+        <v>329</v>
+      </c>
+      <c r="H196" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I196" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A197" t="s">
+        <v>72</v>
+      </c>
+      <c r="B197">
+        <v>2023</v>
+      </c>
+      <c r="C197" t="s">
+        <v>170</v>
+      </c>
+      <c r="D197" t="s">
+        <v>9</v>
+      </c>
+      <c r="F197" t="s">
+        <v>329</v>
+      </c>
+      <c r="H197" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I197" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A198" t="s">
+        <v>72</v>
+      </c>
+      <c r="B198">
+        <v>2023</v>
+      </c>
+      <c r="C198" t="s">
+        <v>170</v>
+      </c>
+      <c r="D198" t="s">
+        <v>9</v>
+      </c>
+      <c r="F198" t="s">
+        <v>329</v>
+      </c>
+      <c r="H198" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I198" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A199" t="s">
+        <v>72</v>
+      </c>
+      <c r="B199">
+        <v>2023</v>
+      </c>
+      <c r="C199" t="s">
+        <v>112</v>
+      </c>
+      <c r="D199" t="s">
+        <v>9</v>
+      </c>
+      <c r="F199" t="s">
+        <v>329</v>
+      </c>
+      <c r="H199" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I199" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A200" t="s">
+        <v>72</v>
+      </c>
+      <c r="B200">
+        <v>2023</v>
+      </c>
+      <c r="C200" t="s">
+        <v>112</v>
+      </c>
+      <c r="D200" t="s">
+        <v>9</v>
+      </c>
+      <c r="F200" t="s">
+        <v>329</v>
+      </c>
+      <c r="H200" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I200" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A201" t="s">
+        <v>72</v>
+      </c>
+      <c r="B201">
+        <v>2023</v>
+      </c>
+      <c r="C201" t="s">
+        <v>47</v>
+      </c>
+      <c r="D201" t="s">
+        <v>15</v>
+      </c>
+      <c r="F201" t="s">
+        <v>329</v>
+      </c>
+      <c r="H201" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I201" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A202" t="s">
+        <v>72</v>
+      </c>
+      <c r="B202">
+        <v>2023</v>
+      </c>
+      <c r="C202" t="s">
+        <v>47</v>
+      </c>
+      <c r="D202" t="s">
+        <v>9</v>
+      </c>
+      <c r="F202" t="s">
+        <v>329</v>
+      </c>
+      <c r="H202" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I202" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A203" t="s">
+        <v>72</v>
+      </c>
+      <c r="B203">
+        <v>2023</v>
+      </c>
+      <c r="C203" t="s">
+        <v>47</v>
+      </c>
+      <c r="D203" t="s">
+        <v>15</v>
+      </c>
+      <c r="F203" t="s">
+        <v>329</v>
+      </c>
+      <c r="H203" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I203" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A204" t="s">
+        <v>72</v>
+      </c>
+      <c r="B204">
+        <v>2023</v>
+      </c>
+      <c r="C204" t="s">
+        <v>170</v>
+      </c>
+      <c r="D204" t="s">
+        <v>9</v>
+      </c>
+      <c r="F204" t="s">
+        <v>329</v>
+      </c>
+      <c r="H204" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I204" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A205" t="s">
+        <v>72</v>
+      </c>
+      <c r="B205">
+        <v>2023</v>
+      </c>
+      <c r="C205" t="s">
+        <v>170</v>
+      </c>
+      <c r="D205" t="s">
+        <v>9</v>
+      </c>
+      <c r="F205" t="s">
+        <v>329</v>
+      </c>
+      <c r="H205" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I205" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A206" t="s">
+        <v>72</v>
+      </c>
+      <c r="B206">
+        <v>2023</v>
+      </c>
+      <c r="C206" t="s">
+        <v>47</v>
+      </c>
+      <c r="D206" t="s">
+        <v>344</v>
+      </c>
+      <c r="F206" t="s">
+        <v>329</v>
+      </c>
+      <c r="H206" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I206" s="4" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A207" t="s">
+        <v>72</v>
+      </c>
+      <c r="B207">
+        <v>2023</v>
+      </c>
+      <c r="C207" t="s">
+        <v>237</v>
+      </c>
+      <c r="D207" t="s">
+        <v>323</v>
+      </c>
+      <c r="F207" t="s">
+        <v>329</v>
+      </c>
+      <c r="H207" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I207" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A208" t="s">
+        <v>72</v>
+      </c>
+      <c r="B208">
+        <v>2023</v>
+      </c>
+      <c r="C208" t="s">
+        <v>170</v>
+      </c>
+      <c r="D208" t="s">
+        <v>323</v>
+      </c>
+      <c r="F208" t="s">
+        <v>329</v>
+      </c>
+      <c r="H208" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I208" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A209" t="s">
+        <v>72</v>
+      </c>
+      <c r="B209">
+        <v>2023</v>
+      </c>
+      <c r="C209" t="s">
+        <v>170</v>
+      </c>
+      <c r="D209" t="s">
+        <v>323</v>
+      </c>
+      <c r="F209" t="s">
+        <v>329</v>
+      </c>
+      <c r="H209" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I209" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A210" t="s">
+        <v>72</v>
+      </c>
+      <c r="B210">
+        <v>2023</v>
+      </c>
+      <c r="C210" t="s">
+        <v>170</v>
+      </c>
+      <c r="D210" t="s">
+        <v>323</v>
+      </c>
+      <c r="F210" t="s">
+        <v>329</v>
+      </c>
+      <c r="H210" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I210" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A211" t="s">
+        <v>72</v>
+      </c>
+      <c r="B211">
+        <v>2023</v>
+      </c>
+      <c r="C211" t="s">
+        <v>49</v>
+      </c>
+      <c r="D211" t="s">
+        <v>15</v>
+      </c>
+      <c r="F211" t="s">
+        <v>329</v>
+      </c>
+      <c r="H211" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I211" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="212" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A212" t="s">
+        <v>72</v>
+      </c>
+      <c r="B212">
+        <v>2023</v>
+      </c>
+      <c r="C212" t="s">
+        <v>112</v>
+      </c>
+      <c r="D212" t="s">
+        <v>15</v>
+      </c>
+      <c r="F212" t="s">
+        <v>329</v>
+      </c>
+      <c r="H212" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I212" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A213" t="s">
+        <v>72</v>
+      </c>
+      <c r="B213">
+        <v>2023</v>
+      </c>
+      <c r="C213" t="s">
+        <v>47</v>
+      </c>
+      <c r="D213" t="s">
+        <v>323</v>
+      </c>
+      <c r="F213" t="s">
+        <v>329</v>
+      </c>
+      <c r="H213" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I213" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="214" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A214" t="s">
+        <v>72</v>
+      </c>
+      <c r="B214">
+        <v>2023</v>
+      </c>
+      <c r="C214" t="s">
+        <v>47</v>
+      </c>
+      <c r="D214" t="s">
+        <v>323</v>
+      </c>
+      <c r="F214" t="s">
+        <v>329</v>
+      </c>
+      <c r="H214" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="I214" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A215" t="s">
+        <v>72</v>
+      </c>
+      <c r="B215">
+        <v>2023</v>
+      </c>
+      <c r="C215" t="s">
+        <v>47</v>
+      </c>
+      <c r="D215" t="s">
+        <v>323</v>
+      </c>
+      <c r="F215" t="s">
+        <v>329</v>
+      </c>
+      <c r="I215" t="s">
+        <v>353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>